<commit_message>
feat(productos): Kit Gestión de Personal y Turnos v2.0 — 9 xlsx regenerados: horas con cruce de medianoche, recargo de convenio en celda (1,25× con nota legal correcta) y contador 80 h/año, las 4 alertas del cuadrante por fórmula (12 h art. 34.3 ET), calendario de vacaciones que cuenta DÍAS con hoja de saldo, coste laboral con SS 33 % en celda y pagas prorrateadas, onboarding 0 % recién descargado con 50 tareas, ficha de evaluación sin #DIV/0!, directorio sin datos de salud (art. 9 RGPD) y vencimientos a 30 empleados, BONUS-02 con 7 FTE y ratio 31,3 %; copy legal corregido (registro horario 2019, LISOS 7.5); fixes del crítico (demos fuera de dl/, CtaFinal 50 tareas, tildes SPA). Censo 0, gate offline 9/9
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-gestion-personal/06-evaluacion-desempeno.xlsx
+++ b/astro-site/public/dl/kit-gestion-personal/06-evaluacion-desempeno.xlsx
@@ -9,10 +9,15 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ficha Evaluación" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ficha (ejemplo relleno)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Histórico'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instrucciones'!$A$1:$B$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Evaluación'!$A$1:$D$50</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Ficha (ejemplo relleno)'!$A$1:$D$50</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Histórico'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Histórico'!$A$1:$G$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,10 +25,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,8 +99,43 @@
       <color rgb="00999999"/>
       <sz val="9"/>
     </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00888888"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +152,21 @@
       <patternFill patternType="solid">
         <fgColor rgb="002D2D2D"/>
         <bgColor rgb="002D2D2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECEFF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002D2D2D"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,7 +240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -221,10 +278,156 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+          <bgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -587,7 +790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -596,7 +799,7 @@
   <sheetData>
     <row r="1"/>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>06 · Evaluación de Desempeño</t>
         </is>
@@ -604,110 +807,201 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Cómo usar esta plantilla:</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>▸ Completa una ficha por empleado y periodo de evaluación.</t>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>▸ La hoja 'Ficha Evaluación' viene EN BLANCO: es el original. Para evaluar a alguien, duplícala (clic derecho sobre la pestaña → Mover o copiar → Crear una copia) y renombra la copia «Apellido-Q3», por ejemplo.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>▸ Puntúa cada competencia de 1 (deficiente) a 5 (excelente).</t>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>▸ La hoja 'Ficha (ejemplo relleno)' es esa misma ficha con un caso real terminado. No la borres: es la referencia de cómo se rellenan las observaciones y el plan de desarrollo.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>▸ La media se calcula automáticamente.</t>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>▸ Puntúa cada competencia de 1 a 5, o elige N/A si no aplica al puesto. La media sale SÓLO de lo valorado y la casilla «Competencias valoradas» te dice sobre cuántas se ha calculado.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>▸ Usa la hoja 'Histórico' para seguir la evolución trimestral.</t>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>▸ Cuando cierres una ficha, copia su PUNTUACIÓN MEDIA a la hoja 'Histórico', en la columna del trimestre que toque.</t>
         </is>
       </c>
     </row>
     <row r="9"/>
     <row r="10">
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Escala de puntuación:</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>▸ 1 = Deficiente — No cumple requisitos mínimos</t>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>▸ 1 = Deficiente — No cumple los requisitos mínimos del puesto</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>▸ 2 = Mejorable — Cumple parcialmente, necesita supervisión constante</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>▸ 3 = Adecuado — Cumple lo esperado para el puesto</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>▸ 4 = Bueno — Supera expectativas en varias áreas</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>▸ 5 = Excelente — Referencia para el equipo</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
+    <row r="16">
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>▸ N/A = No aplica al puesto. No es un cero: queda fuera de la media.</t>
+        </is>
+      </c>
+    </row>
     <row r="17">
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>Nota media y nivel:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>▸ Con la ficha recién abierta, la media y el nivel están EN BLANCO. Es lo correcto: un empleado sin puntuar no tiene nota, y la ficha se imprime y se firma tal cual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>▸ El nivel se colorea solo: verde a partir de 3,5, ámbar entre 1,5 y 3,5 y rojo por debajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>Histórico y tendencia:</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>▸ La columna Tendencia compara los DOS ÚLTIMOS trimestres informados, no sólo Q4 contra Q3: con Q1 y Q2 rellenos ya dice algo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>▸ Rellena los trimestres de izquierda a derecha (Q1, luego Q2…): la comparación cuenta cuántas notas hay, no en qué columna están.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>Plan de desarrollo individual:</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>▸ El bloque del final de la ficha es lo que convierte una evaluación en una mejora: acción formativa, fecha objetivo y quién responde de que ocurra, con un indicador que se pueda comprobar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>▸ Revísalo en la evaluación siguiente antes de puntuar nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="B30" s="24" t="inlineStr">
         <is>
           <t>Frecuencia recomendada:</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="3" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="24" t="inlineStr">
         <is>
           <t>▸ Evaluación formal cada 3 meses (trimestral).</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="24" t="inlineStr">
         <is>
           <t>▸ Feedback informal continuo — al menos 1 conversación/semana.</t>
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-gestion-personal · info@aichef.pro</t>
+    <row r="33"/>
+    <row r="34">
+      <c r="B34" s="25" t="inlineStr">
+        <is>
+          <t>Para editar una celda bloqueada: Revisar → Desproteger hoja (no tiene contraseña). Las celdas verdes ya son editables sin desproteger nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="25" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="25" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/kit-gestion-personal · info@aichef.pro</t>
         </is>
       </c>
     </row>
@@ -732,370 +1026,539 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Ficha de Evaluación de Desempeño</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>AI Chef Pro · aichef.pro — Kit Gestión de Personal y Turnos</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
+    <row r="3">
+      <c r="A3" s="28" t="n"/>
+      <c r="B3" s="28" t="n"/>
+      <c r="C3" s="28" t="n"/>
+      <c r="D3" s="28" t="n"/>
+    </row>
     <row r="4">
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="28" t="n"/>
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Empleado:</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
+      <c r="C4" s="30" t="n"/>
       <c r="D4" s="8" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="6" t="inlineStr">
+      <c r="A5" s="28" t="n"/>
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Puesto:</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
+      <c r="C5" s="30" t="n"/>
       <c r="D5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="A6" s="28" t="n"/>
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>Periodo evaluado:</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n"/>
+      <c r="C6" s="30" t="n"/>
       <c r="D6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="6" t="inlineStr">
+      <c r="A7" s="28" t="n"/>
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Evaluador:</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
+      <c r="C7" s="30" t="n"/>
       <c r="D7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="A8" s="28" t="n"/>
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>Fecha evaluación:</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
+      <c r="C8" s="31" t="n"/>
       <c r="D8" s="8" t="n"/>
     </row>
-    <row r="9"/>
+    <row r="9">
+      <c r="A9" s="28" t="n"/>
+      <c r="B9" s="28" t="n"/>
+      <c r="C9" s="28" t="n"/>
+      <c r="D9" s="28" t="n"/>
+    </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>COMPETENCIAS (puntúa 1-5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
+        <is>
+          <t>COMPETENCIAS — puntúa de 1 a 5, o N/A si la competencia no aplica al puesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="33" t="inlineStr">
         <is>
           <t>Competencia</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="33" t="inlineStr">
         <is>
           <t>Puntuación (1-5)</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="33" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="11" t="n">
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>Puntualidad y asistencia</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="14" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="C12" s="36" t="n"/>
+      <c r="D12" s="30" t="n"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="35" t="inlineStr">
         <is>
           <t>Presentación personal e higiene</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="14" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="C13" s="36" t="n"/>
+      <c r="D13" s="30" t="n"/>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>Trabajo en equipo y colaboración</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="14" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="C14" s="36" t="n"/>
+      <c r="D14" s="30" t="n"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="34" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>Iniciativa y proactividad</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n"/>
-      <c r="D15" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="n">
+      <c r="C15" s="36" t="n"/>
+      <c r="D15" s="30" t="n"/>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="35" t="inlineStr">
         <is>
           <t>Limpieza y orden del puesto</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n"/>
-      <c r="D16" s="14" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="n">
+      <c r="C16" s="36" t="n"/>
+      <c r="D16" s="30" t="n"/>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="34" t="n">
         <v>6</v>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>Rapidez y eficiencia</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="14" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="n">
+      <c r="C17" s="36" t="n"/>
+      <c r="D17" s="30" t="n"/>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="34" t="n">
         <v>7</v>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="35" t="inlineStr">
         <is>
           <t>Atención al cliente</t>
         </is>
       </c>
-      <c r="C18" s="13" t="n"/>
-      <c r="D18" s="14" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="n">
+      <c r="C18" s="36" t="n"/>
+      <c r="D18" s="30" t="n"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="34" t="n">
         <v>8</v>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>Conocimiento de la carta / producto</t>
         </is>
       </c>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="14" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="n">
+      <c r="C19" s="36" t="n"/>
+      <c r="D19" s="30" t="n"/>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="34" t="n">
         <v>9</v>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="35" t="inlineStr">
         <is>
           <t>Gestión del estrés en servicio</t>
         </is>
       </c>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="14" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="n">
+      <c r="C20" s="36" t="n"/>
+      <c r="D20" s="30" t="n"/>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="35" t="inlineStr">
         <is>
           <t>Comunicación con compañeros y superiores</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n"/>
-      <c r="D21" s="14" t="n"/>
+      <c r="C21" s="36" t="n"/>
+      <c r="D21" s="30" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="n"/>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="A22" s="37" t="n"/>
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>PUNTUACIÓN MEDIA</t>
         </is>
       </c>
-      <c r="C22" s="17" t="str">
-        <f>AVERAGE(C12:C21)</f>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="C22" s="39">
+        <f>IF(COUNT($C$12:$C$21)=0,"",ROUND(AVERAGE($C$12:$C$21),2))</f>
+        <v/>
+      </c>
+      <c r="D22" s="28" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="16" t="inlineStr">
+      <c r="A23" s="28" t="n"/>
+      <c r="B23" s="38" t="inlineStr">
         <is>
           <t>NIVEL</t>
         </is>
       </c>
-      <c r="C23" s="18" t="str">
-        <f>IF(C22&gt;=4.5,"⭐ EXCELENTE",IF(C22&gt;=3.5,"✓ BUENO",IF(C22&gt;=2.5,"→ ADECUADO",IF(C22&gt;=1.5,"⚠ MEJORABLE","✗ DEFICIENTE"))))</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="24"/>
+      <c r="C23" s="40" t="str">
+        <f>IF(COUNT($C$12:$C$21)&lt;5,"⚠ puntúa al menos 5 competencias",IF($C$22="","",IF($C$22&gt;=4.5,"⭐ EXCELENTE",IF($C$22&gt;=3.5,"✓ BUENO",IF($C$22&gt;=2.5,"→ ADECUADO",IF($C$22&gt;=1.5,"⚠ MEJORABLE","✗ DEFICIENTE"))))))</f>
+        <v>⚠ puntúa al menos 5 competencias</v>
+      </c>
+      <c r="D23" s="28" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="28" t="n"/>
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>Competencias valoradas</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="str">
+        <f>COUNT($C$12:$C$21)&amp;" de 10"</f>
+        <v>0 de 10</v>
+      </c>
+      <c r="D24" s="42" t="inlineStr">
+        <is>
+          <t>← las N/A no cuentan: la media sale sólo de las competencias puntuadas</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="28" t="n"/>
+      <c r="B25" s="28" t="n"/>
+      <c r="C25" s="28" t="n"/>
+      <c r="D25" s="28" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t>FORTALEZAS DESTACADAS</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="22" t="n"/>
-      <c r="D26" s="8" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="7" t="n"/>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="43" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B27" s="44" t="n"/>
       <c r="C27" s="22" t="n"/>
       <c r="D27" s="8" t="n"/>
     </row>
-    <row r="28">
-      <c r="B28" s="7" t="n"/>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="43" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B28" s="44" t="n"/>
       <c r="C28" s="22" t="n"/>
       <c r="D28" s="8" t="n"/>
     </row>
-    <row r="29"/>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="43" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B29" s="45" t="n"/>
+    </row>
     <row r="30">
-      <c r="A30" s="9" t="inlineStr">
+      <c r="A30" s="28" t="n"/>
+      <c r="B30" s="28" t="n"/>
+      <c r="C30" s="28" t="n"/>
+      <c r="D30" s="28" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="32" t="inlineStr">
         <is>
           <t>ÁREAS DE MEJORA</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="22" t="n"/>
-      <c r="D31" s="8" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="7" t="n"/>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="43" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B32" s="44" t="n"/>
       <c r="C32" s="22" t="n"/>
       <c r="D32" s="8" t="n"/>
     </row>
-    <row r="33">
-      <c r="B33" s="7" t="n"/>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="43" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B33" s="44" t="n"/>
       <c r="C33" s="22" t="n"/>
       <c r="D33" s="8" t="n"/>
     </row>
-    <row r="34"/>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="43" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B34" s="45" t="n"/>
+    </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>OBJETIVOS PARA PRÓXIMO PERIODO</t>
-        </is>
-      </c>
+      <c r="A35" s="28" t="n"/>
+      <c r="B35" s="28" t="n"/>
+      <c r="C35" s="28" t="n"/>
+      <c r="D35" s="28" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="22" t="n"/>
-      <c r="D36" s="8" t="n"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="7" t="n"/>
+      <c r="A36" s="32" t="inlineStr">
+        <is>
+          <t>OBJETIVOS PARA EL PRÓXIMO PERIODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="43" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B37" s="44" t="n"/>
       <c r="C37" s="22" t="n"/>
       <c r="D37" s="8" t="n"/>
     </row>
-    <row r="38">
-      <c r="B38" s="7" t="n"/>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="43" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B38" s="44" t="n"/>
       <c r="C38" s="22" t="n"/>
       <c r="D38" s="8" t="n"/>
     </row>
-    <row r="39"/>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="43" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B39" s="45" t="n"/>
+    </row>
     <row r="40">
-      <c r="A40" s="19" t="inlineStr">
-        <is>
-          <t>Firma evaluador: _________________     Firma empleado: _________________</t>
-        </is>
-      </c>
+      <c r="A40" s="28" t="n"/>
+      <c r="B40" s="28" t="n"/>
+      <c r="C40" s="28" t="n"/>
+      <c r="D40" s="28" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="inlineStr">
+      <c r="A41" s="32" t="inlineStr">
+        <is>
+          <t>PLAN DE DESARROLLO INDIVIDUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="46" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t>Acción formativa</t>
+        </is>
+      </c>
+      <c r="C42" s="46" t="inlineStr">
+        <is>
+          <t>Fecha objetivo</t>
+        </is>
+      </c>
+      <c r="D42" s="46" t="inlineStr">
+        <is>
+          <t>Responsable e indicador de logro</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" s="45" t="n"/>
+      <c r="C43" s="47" t="n"/>
+      <c r="D43" s="45" t="n"/>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" s="49" t="n"/>
+      <c r="C44" s="50" t="n"/>
+      <c r="D44" s="49" t="n"/>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="B45" s="49" t="n"/>
+      <c r="C45" s="50" t="n"/>
+      <c r="D45" s="49" t="n"/>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Firma evaluador: _________________          Firma empleado: _________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Fecha: ___/___/______</t>
         </is>
       </c>
     </row>
-    <row r="42"/>
-    <row r="43">
-      <c r="A43" s="19" t="inlineStr">
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="51" t="inlineStr">
         <is>
           <t>© 2026 AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="24">
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="B29:D29"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A50:D50"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="B34:D34"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A43:D43"/>
     <mergeCell ref="C7:D7"/>
+    <mergeCell ref="A26:D26"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B37:D37"/>
+    <mergeCell ref="A36:D36"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B39:D39"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="C8:D8"/>
-    <mergeCell ref="B31:D31"/>
     <mergeCell ref="B33:D33"/>
-    <mergeCell ref="A25:D25"/>
   </mergeCells>
+  <conditionalFormatting sqref="C23">
+    <cfRule type="containsText" priority="1" operator="containsText" dxfId="0" stopIfTrue="1" text="DEFICIENTE">
+      <formula>NOT(ISERROR(SEARCH("DEFICIENTE",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="2" operator="containsText" dxfId="1" stopIfTrue="1" text="MEJORABLE">
+      <formula>NOT(ISERROR(SEARCH("MEJORABLE",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="3" operator="containsText" dxfId="1" stopIfTrue="1" text="ADECUADO">
+      <formula>NOT(ISERROR(SEARCH("ADECUADO",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="4" operator="containsText" dxfId="2" stopIfTrue="1" text="EXCELENTE">
+      <formula>NOT(ISERROR(SEARCH("EXCELENTE",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="5" operator="containsText" dxfId="2" stopIfTrue="1" text="BUENO">
+      <formula>NOT(ISERROR(SEARCH("BUENO",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="6" operator="containsText" dxfId="1" stopIfTrue="1" text="puntúa al menos">
+      <formula>NOT(ISERROR(SEARCH("puntúa al menos",C23)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C12 C13 C14 C15 C16 C17 C18 C19 C20 C21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Introduce un valor entre 1 y 5" prompt="1=Deficiente, 2=Mejorable, 3=Adecuado, 4=Bueno, 5=Excelente" type="whole" operator="between">
-      <formula1>1</formula1>
-      <formula2>5</formula2>
+    <dataValidation sqref="C12:C21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Puntuación no válida" error="Escribe 1, 2, 3, 4, 5 o N/A." promptTitle="kitgp-v2c · Puntuación no válida" prompt="1 = Deficiente · 2 = Mejorable · 3 = Adecuado · 4 = Bueno · 5 = Excelente. Elige N/A cuando la competencia no aplique al puesto (un cocinero de partida no atiende sala): la media se calcula SÓLO con lo valorado, así que N/A no penaliza." type="list" errorStyle="stop">
+      <formula1>"1,2,3,4,5,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
@@ -1114,313 +1577,1196 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>Ficha de Evaluación de Desempeño — EJEMPLO RELLENO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>AI Chef Pro · aichef.pro — Kit Gestión de Personal y Turnos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>Empleado:</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>Marta Ruiz Beltrán</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>Puesto:</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>Jefa de partida — cuarto frío</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>Periodo evaluado:</t>
+        </is>
+      </c>
+      <c r="C6" s="52" t="inlineStr">
+        <is>
+          <t>Q3 2026 (julio-septiembre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>Evaluador:</t>
+        </is>
+      </c>
+      <c r="C7" s="52" t="inlineStr">
+        <is>
+          <t>John Guerrero — jefe de cocina</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>Fecha evaluación:</t>
+        </is>
+      </c>
+      <c r="C8" s="53" t="n">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="32" t="inlineStr">
+        <is>
+          <t>COMPETENCIAS — puntúa de 1 a 5, o N/A si la competencia no aplica al puesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>Competencia</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>Puntuación (1-5)</t>
+        </is>
+      </c>
+      <c r="D11" s="46" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="54" t="inlineStr">
+        <is>
+          <t>Puntualidad y asistencia</t>
+        </is>
+      </c>
+      <c r="C12" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
+        <is>
+          <t>Ni un retraso en el trimestre; avisó con 48 h del único cambio de turno que pidió.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="54" t="inlineStr">
+        <is>
+          <t>Presentación personal e higiene</t>
+        </is>
+      </c>
+      <c r="C13" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="54" t="inlineStr">
+        <is>
+          <t>Uniforme y aseo impecables; corrige a los ayudantes cuando se saltan el gorro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="54" t="inlineStr">
+        <is>
+          <t>Trabajo en equipo y colaboración</t>
+        </is>
+      </c>
+      <c r="C14" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="54" t="inlineStr">
+        <is>
+          <t>Se lleva bien con pase y con sala; en el cambio de carta tiró del equipo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="54" t="inlineStr">
+        <is>
+          <t>Iniciativa y proactividad</t>
+        </is>
+      </c>
+      <c r="C15" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>Propuso el escandallo del steak tartar y bajó la merma del salmón un 6 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="54" t="inlineStr">
+        <is>
+          <t>Limpieza y orden del puesto</t>
+        </is>
+      </c>
+      <c r="C16" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="54" t="inlineStr">
+        <is>
+          <t>Cuarto frío cierra siempre en orden; los registros APPCC al día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="48" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="54" t="inlineStr">
+        <is>
+          <t>Rapidez y eficiencia</t>
+        </is>
+      </c>
+      <c r="C17" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="54" t="inlineStr">
+        <is>
+          <t>Va sobrada en producción; se atasca cuando entran dos comandas de tartar seguidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="48" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" s="54" t="inlineStr">
+        <is>
+          <t>Atención al cliente</t>
+        </is>
+      </c>
+      <c r="C18" s="48" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D18" s="54" t="inlineStr">
+        <is>
+          <t>No aplica: no atiende sala en este puesto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="B19" s="54" t="inlineStr">
+        <is>
+          <t>Conocimiento de la carta / producto</t>
+        </is>
+      </c>
+      <c r="C19" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="54" t="inlineStr">
+        <is>
+          <t>Domina su partida; le falta soltura con la bodega y los postres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="48" t="n">
+        <v>9</v>
+      </c>
+      <c r="B20" s="54" t="inlineStr">
+        <is>
+          <t>Gestión del estrés en servicio</t>
+        </is>
+      </c>
+      <c r="C20" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="54" t="inlineStr">
+        <is>
+          <t>En los servicios de más de 90 cubiertos pierde el orden de los pases. Es el punto a trabajar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" s="54" t="inlineStr">
+        <is>
+          <t>Comunicación con compañeros y superiores</t>
+        </is>
+      </c>
+      <c r="C21" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="54" t="inlineStr">
+        <is>
+          <t>Pregunta lo que no sabe y da parte de las incidencias por escrito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>PUNTUACIÓN MEDIA</t>
+        </is>
+      </c>
+      <c r="C22" s="55">
+        <f>IF(COUNT($C$12:$C$21)=0,"",ROUND(AVERAGE($C$12:$C$21),2))</f>
+        <v>4.22</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>NIVEL</t>
+        </is>
+      </c>
+      <c r="C23" s="56" t="str">
+        <f>IF(COUNT($C$12:$C$21)&lt;5,"⚠ puntúa al menos 5 competencias",IF($C$22="","",IF($C$22&gt;=4.5,"⭐ EXCELENTE",IF($C$22&gt;=3.5,"✓ BUENO",IF($C$22&gt;=2.5,"→ ADECUADO",IF($C$22&gt;=1.5,"⚠ MEJORABLE","✗ DEFICIENTE"))))))</f>
+        <v>✓ BUENO</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Competencias valoradas</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="str">
+        <f>COUNT($C$12:$C$21)&amp;" de 10"</f>
+        <v>9 de 10</v>
+      </c>
+      <c r="D24" s="42" t="inlineStr">
+        <is>
+          <t>← las N/A no cuentan: la media sale sólo de las competencias puntuadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="32" t="inlineStr">
+        <is>
+          <t>FORTALEZAS DESTACADAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="48" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
+        <is>
+          <t>Organización y limpieza del cuarto frío: la partida mejor llevada del equipo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="48" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>Muy fiable con el producto: cero mermas por mala conservación en todo el trimestre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="48" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>Formadora natural — los dos ayudantes nuevos aprendieron con ella.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>ÁREAS DE MEJORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="48" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>Gestión del estrés cuando se juntan dos comandas de tartar en el mismo pase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="48" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Conocimiento de bodega y de la partida de postres, que hoy no cubre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="48" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="n"/>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
+          <t>OBJETIVOS PARA EL PRÓXIMO PERIODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="48" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>Cubrir la partida de postres dos servicios por semana a partir de noviembre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="48" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>Sacar adelante 4 servicios de más de 90 cubiertos sin retrasos en el pase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="48" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="n"/>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="32" t="inlineStr">
+        <is>
+          <t>PLAN DE DESARROLLO INDIVIDUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="46" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t>Acción formativa</t>
+        </is>
+      </c>
+      <c r="C42" s="46" t="inlineStr">
+        <is>
+          <t>Fecha objetivo</t>
+        </is>
+      </c>
+      <c r="D42" s="46" t="inlineStr">
+        <is>
+          <t>Responsable e indicador de logro</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>Curso interno de organización de partida en servicio alto (8 h, dos sesiones)</t>
+        </is>
+      </c>
+      <c r="C43" s="50" t="n">
+        <v>46341</v>
+      </c>
+      <c r="D43" s="49" t="inlineStr">
+        <is>
+          <t>Jefe de cocina · 4 servicios de +90 cubiertos sin retraso en el pase</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" s="49" t="inlineStr">
+        <is>
+          <t>Rotación de dos servicios semanales en la partida de postres</t>
+        </is>
+      </c>
+      <c r="C44" s="50" t="n">
+        <v>46376</v>
+      </c>
+      <c r="D44" s="49" t="inlineStr">
+        <is>
+          <t>Jefa de pastelería · saca la carta de postres sin apoyo</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="B45" s="49" t="n"/>
+      <c r="C45" s="50" t="n"/>
+      <c r="D45" s="49" t="n"/>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Firma evaluador: _________________          Firma empleado: _________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Fecha: ___/___/______</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="51" t="inlineStr">
+        <is>
+          <t>© 2026 AI Chef Pro · aichef.pro</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="24">
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="C8:D8"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C23">
+    <cfRule type="containsText" priority="1" operator="containsText" dxfId="0" stopIfTrue="1" text="DEFICIENTE">
+      <formula>NOT(ISERROR(SEARCH("DEFICIENTE",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="2" operator="containsText" dxfId="1" stopIfTrue="1" text="MEJORABLE">
+      <formula>NOT(ISERROR(SEARCH("MEJORABLE",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="3" operator="containsText" dxfId="1" stopIfTrue="1" text="ADECUADO">
+      <formula>NOT(ISERROR(SEARCH("ADECUADO",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="4" operator="containsText" dxfId="2" stopIfTrue="1" text="EXCELENTE">
+      <formula>NOT(ISERROR(SEARCH("EXCELENTE",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="5" operator="containsText" dxfId="2" stopIfTrue="1" text="BUENO">
+      <formula>NOT(ISERROR(SEARCH("BUENO",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="6" operator="containsText" dxfId="1" stopIfTrue="1" text="puntúa al menos">
+      <formula>NOT(ISERROR(SEARCH("puntúa al menos",C23)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="C12:C21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Puntuación no válida" error="Escribe 1, 2, 3, 4, 5 o N/A." promptTitle="kitgp-v2c · Puntuación no válida" prompt="1 = Deficiente · 2 = Mejorable · 3 = Adecuado · 4 = Bueno · 5 = Excelente. Elige N/A cuando la competencia no aplique al puesto (un cocinero de partida no atiende sala): la media se calcula SÓLO con lo valorado, así que N/A no penaliza." type="list" errorStyle="stop">
+      <formula1>"1,2,3,4,5,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="004A148C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Histórico de Evaluaciones</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>AI Chef Pro · aichef.pro — Kit Gestión de Personal y Turnos</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="28" t="n"/>
+      <c r="B3" s="28" t="n"/>
+      <c r="C3" s="28" t="n"/>
+      <c r="D3" s="28" t="n"/>
+      <c r="E3" s="28" t="n"/>
+      <c r="F3" s="28" t="n"/>
+      <c r="G3" s="28" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="33" t="inlineStr">
         <is>
           <t>Empleado</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="33" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="33" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="33" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="33" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="33" t="inlineStr">
         <is>
           <t>Media Anual</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="G4" s="33" t="inlineStr">
         <is>
           <t>Tendencia</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="n"/>
-      <c r="B5" s="21" t="n"/>
-      <c r="C5" s="21" t="n"/>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="21" t="n"/>
-      <c r="F5" s="17">
-        <f>IF(COUNT(B5:E5)&gt;0,AVERAGE(B5:E5),"")</f>
-        <v/>
-      </c>
-      <c r="G5" s="11">
-        <f>IF(AND(E5&lt;&gt;"",D5&lt;&gt;""),IF(E5&gt;D5,"↑ Mejora",IF(E5&lt;D5,"↓ Baja","→ Estable")),"")</f>
+      <c r="A5" s="30" t="n"/>
+      <c r="B5" s="57" t="n"/>
+      <c r="C5" s="57" t="n"/>
+      <c r="D5" s="57" t="n"/>
+      <c r="E5" s="57" t="n"/>
+      <c r="F5" s="58">
+        <f>IF(COUNT($B5:$E5)=0,"",ROUND(AVERAGE($B5:$E5),2))</f>
+        <v/>
+      </c>
+      <c r="G5" s="34">
+        <f>IF(COUNT($B5:$E5)&lt;2,"",IF(IF($E5&lt;&gt;"",$E5,IF($D5&lt;&gt;"",$D5,IF($C5&lt;&gt;"",$C5,$B5)))&gt;IF($E5&lt;&gt;"",IF($D5&lt;&gt;"",$D5,IF($C5&lt;&gt;"",$C5,$B5)),IF($D5&lt;&gt;"",IF($C5&lt;&gt;"",$C5,$B5),IF($C5&lt;&gt;"",$B5,""))),"↑ Mejora",IF(IF($E5&lt;&gt;"",$E5,IF($D5&lt;&gt;"",$D5,IF($C5&lt;&gt;"",$C5,$B5)))&lt;IF($E5&lt;&gt;"",IF($D5&lt;&gt;"",$D5,IF($C5&lt;&gt;"",$C5,$B5)),IF($D5&lt;&gt;"",IF($C5&lt;&gt;"",$C5,$B5),IF($C5&lt;&gt;"",$B5,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="n"/>
-      <c r="B6" s="21" t="n"/>
-      <c r="C6" s="21" t="n"/>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="21" t="n"/>
-      <c r="F6" s="17">
-        <f>IF(COUNT(B6:E6)&gt;0,AVERAGE(B6:E6),"")</f>
-        <v/>
-      </c>
-      <c r="G6" s="11">
-        <f>IF(AND(E6&lt;&gt;"",D6&lt;&gt;""),IF(E6&gt;D6,"↑ Mejora",IF(E6&lt;D6,"↓ Baja","→ Estable")),"")</f>
+      <c r="A6" s="30" t="n"/>
+      <c r="B6" s="57" t="n"/>
+      <c r="C6" s="57" t="n"/>
+      <c r="D6" s="57" t="n"/>
+      <c r="E6" s="57" t="n"/>
+      <c r="F6" s="58">
+        <f>IF(COUNT($B6:$E6)=0,"",ROUND(AVERAGE($B6:$E6),2))</f>
+        <v/>
+      </c>
+      <c r="G6" s="34">
+        <f>IF(COUNT($B6:$E6)&lt;2,"",IF(IF($E6&lt;&gt;"",$E6,IF($D6&lt;&gt;"",$D6,IF($C6&lt;&gt;"",$C6,$B6)))&gt;IF($E6&lt;&gt;"",IF($D6&lt;&gt;"",$D6,IF($C6&lt;&gt;"",$C6,$B6)),IF($D6&lt;&gt;"",IF($C6&lt;&gt;"",$C6,$B6),IF($C6&lt;&gt;"",$B6,""))),"↑ Mejora",IF(IF($E6&lt;&gt;"",$E6,IF($D6&lt;&gt;"",$D6,IF($C6&lt;&gt;"",$C6,$B6)))&lt;IF($E6&lt;&gt;"",IF($D6&lt;&gt;"",$D6,IF($C6&lt;&gt;"",$C6,$B6)),IF($D6&lt;&gt;"",IF($C6&lt;&gt;"",$C6,$B6),IF($C6&lt;&gt;"",$B6,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="n"/>
-      <c r="B7" s="21" t="n"/>
-      <c r="C7" s="21" t="n"/>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="21" t="n"/>
-      <c r="F7" s="17">
-        <f>IF(COUNT(B7:E7)&gt;0,AVERAGE(B7:E7),"")</f>
-        <v/>
-      </c>
-      <c r="G7" s="11">
-        <f>IF(AND(E7&lt;&gt;"",D7&lt;&gt;""),IF(E7&gt;D7,"↑ Mejora",IF(E7&lt;D7,"↓ Baja","→ Estable")),"")</f>
+      <c r="A7" s="30" t="n"/>
+      <c r="B7" s="57" t="n"/>
+      <c r="C7" s="57" t="n"/>
+      <c r="D7" s="57" t="n"/>
+      <c r="E7" s="57" t="n"/>
+      <c r="F7" s="58">
+        <f>IF(COUNT($B7:$E7)=0,"",ROUND(AVERAGE($B7:$E7),2))</f>
+        <v/>
+      </c>
+      <c r="G7" s="34">
+        <f>IF(COUNT($B7:$E7)&lt;2,"",IF(IF($E7&lt;&gt;"",$E7,IF($D7&lt;&gt;"",$D7,IF($C7&lt;&gt;"",$C7,$B7)))&gt;IF($E7&lt;&gt;"",IF($D7&lt;&gt;"",$D7,IF($C7&lt;&gt;"",$C7,$B7)),IF($D7&lt;&gt;"",IF($C7&lt;&gt;"",$C7,$B7),IF($C7&lt;&gt;"",$B7,""))),"↑ Mejora",IF(IF($E7&lt;&gt;"",$E7,IF($D7&lt;&gt;"",$D7,IF($C7&lt;&gt;"",$C7,$B7)))&lt;IF($E7&lt;&gt;"",IF($D7&lt;&gt;"",$D7,IF($C7&lt;&gt;"",$C7,$B7)),IF($D7&lt;&gt;"",IF($C7&lt;&gt;"",$C7,$B7),IF($C7&lt;&gt;"",$B7,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="n"/>
-      <c r="B8" s="21" t="n"/>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="21" t="n"/>
-      <c r="F8" s="17">
-        <f>IF(COUNT(B8:E8)&gt;0,AVERAGE(B8:E8),"")</f>
-        <v/>
-      </c>
-      <c r="G8" s="11">
-        <f>IF(AND(E8&lt;&gt;"",D8&lt;&gt;""),IF(E8&gt;D8,"↑ Mejora",IF(E8&lt;D8,"↓ Baja","→ Estable")),"")</f>
+      <c r="A8" s="30" t="n"/>
+      <c r="B8" s="57" t="n"/>
+      <c r="C8" s="57" t="n"/>
+      <c r="D8" s="57" t="n"/>
+      <c r="E8" s="57" t="n"/>
+      <c r="F8" s="58">
+        <f>IF(COUNT($B8:$E8)=0,"",ROUND(AVERAGE($B8:$E8),2))</f>
+        <v/>
+      </c>
+      <c r="G8" s="34">
+        <f>IF(COUNT($B8:$E8)&lt;2,"",IF(IF($E8&lt;&gt;"",$E8,IF($D8&lt;&gt;"",$D8,IF($C8&lt;&gt;"",$C8,$B8)))&gt;IF($E8&lt;&gt;"",IF($D8&lt;&gt;"",$D8,IF($C8&lt;&gt;"",$C8,$B8)),IF($D8&lt;&gt;"",IF($C8&lt;&gt;"",$C8,$B8),IF($C8&lt;&gt;"",$B8,""))),"↑ Mejora",IF(IF($E8&lt;&gt;"",$E8,IF($D8&lt;&gt;"",$D8,IF($C8&lt;&gt;"",$C8,$B8)))&lt;IF($E8&lt;&gt;"",IF($D8&lt;&gt;"",$D8,IF($C8&lt;&gt;"",$C8,$B8)),IF($D8&lt;&gt;"",IF($C8&lt;&gt;"",$C8,$B8),IF($C8&lt;&gt;"",$B8,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="n"/>
-      <c r="B9" s="21" t="n"/>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="21" t="n"/>
-      <c r="F9" s="17">
-        <f>IF(COUNT(B9:E9)&gt;0,AVERAGE(B9:E9),"")</f>
-        <v/>
-      </c>
-      <c r="G9" s="11">
-        <f>IF(AND(E9&lt;&gt;"",D9&lt;&gt;""),IF(E9&gt;D9,"↑ Mejora",IF(E9&lt;D9,"↓ Baja","→ Estable")),"")</f>
+      <c r="A9" s="30" t="n"/>
+      <c r="B9" s="57" t="n"/>
+      <c r="C9" s="57" t="n"/>
+      <c r="D9" s="57" t="n"/>
+      <c r="E9" s="57" t="n"/>
+      <c r="F9" s="58">
+        <f>IF(COUNT($B9:$E9)=0,"",ROUND(AVERAGE($B9:$E9),2))</f>
+        <v/>
+      </c>
+      <c r="G9" s="34">
+        <f>IF(COUNT($B9:$E9)&lt;2,"",IF(IF($E9&lt;&gt;"",$E9,IF($D9&lt;&gt;"",$D9,IF($C9&lt;&gt;"",$C9,$B9)))&gt;IF($E9&lt;&gt;"",IF($D9&lt;&gt;"",$D9,IF($C9&lt;&gt;"",$C9,$B9)),IF($D9&lt;&gt;"",IF($C9&lt;&gt;"",$C9,$B9),IF($C9&lt;&gt;"",$B9,""))),"↑ Mejora",IF(IF($E9&lt;&gt;"",$E9,IF($D9&lt;&gt;"",$D9,IF($C9&lt;&gt;"",$C9,$B9)))&lt;IF($E9&lt;&gt;"",IF($D9&lt;&gt;"",$D9,IF($C9&lt;&gt;"",$C9,$B9)),IF($D9&lt;&gt;"",IF($C9&lt;&gt;"",$C9,$B9),IF($C9&lt;&gt;"",$B9,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="21" t="n"/>
-      <c r="C10" s="21" t="n"/>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="17">
-        <f>IF(COUNT(B10:E10)&gt;0,AVERAGE(B10:E10),"")</f>
-        <v/>
-      </c>
-      <c r="G10" s="11">
-        <f>IF(AND(E10&lt;&gt;"",D10&lt;&gt;""),IF(E10&gt;D10,"↑ Mejora",IF(E10&lt;D10,"↓ Baja","→ Estable")),"")</f>
+      <c r="A10" s="30" t="n"/>
+      <c r="B10" s="57" t="n"/>
+      <c r="C10" s="57" t="n"/>
+      <c r="D10" s="57" t="n"/>
+      <c r="E10" s="57" t="n"/>
+      <c r="F10" s="58">
+        <f>IF(COUNT($B10:$E10)=0,"",ROUND(AVERAGE($B10:$E10),2))</f>
+        <v/>
+      </c>
+      <c r="G10" s="34">
+        <f>IF(COUNT($B10:$E10)&lt;2,"",IF(IF($E10&lt;&gt;"",$E10,IF($D10&lt;&gt;"",$D10,IF($C10&lt;&gt;"",$C10,$B10)))&gt;IF($E10&lt;&gt;"",IF($D10&lt;&gt;"",$D10,IF($C10&lt;&gt;"",$C10,$B10)),IF($D10&lt;&gt;"",IF($C10&lt;&gt;"",$C10,$B10),IF($C10&lt;&gt;"",$B10,""))),"↑ Mejora",IF(IF($E10&lt;&gt;"",$E10,IF($D10&lt;&gt;"",$D10,IF($C10&lt;&gt;"",$C10,$B10)))&lt;IF($E10&lt;&gt;"",IF($D10&lt;&gt;"",$D10,IF($C10&lt;&gt;"",$C10,$B10)),IF($D10&lt;&gt;"",IF($C10&lt;&gt;"",$C10,$B10),IF($C10&lt;&gt;"",$B10,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="n"/>
-      <c r="B11" s="21" t="n"/>
-      <c r="C11" s="21" t="n"/>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="21" t="n"/>
-      <c r="F11" s="17">
-        <f>IF(COUNT(B11:E11)&gt;0,AVERAGE(B11:E11),"")</f>
-        <v/>
-      </c>
-      <c r="G11" s="11">
-        <f>IF(AND(E11&lt;&gt;"",D11&lt;&gt;""),IF(E11&gt;D11,"↑ Mejora",IF(E11&lt;D11,"↓ Baja","→ Estable")),"")</f>
+      <c r="A11" s="30" t="n"/>
+      <c r="B11" s="57" t="n"/>
+      <c r="C11" s="57" t="n"/>
+      <c r="D11" s="57" t="n"/>
+      <c r="E11" s="57" t="n"/>
+      <c r="F11" s="58">
+        <f>IF(COUNT($B11:$E11)=0,"",ROUND(AVERAGE($B11:$E11),2))</f>
+        <v/>
+      </c>
+      <c r="G11" s="34">
+        <f>IF(COUNT($B11:$E11)&lt;2,"",IF(IF($E11&lt;&gt;"",$E11,IF($D11&lt;&gt;"",$D11,IF($C11&lt;&gt;"",$C11,$B11)))&gt;IF($E11&lt;&gt;"",IF($D11&lt;&gt;"",$D11,IF($C11&lt;&gt;"",$C11,$B11)),IF($D11&lt;&gt;"",IF($C11&lt;&gt;"",$C11,$B11),IF($C11&lt;&gt;"",$B11,""))),"↑ Mejora",IF(IF($E11&lt;&gt;"",$E11,IF($D11&lt;&gt;"",$D11,IF($C11&lt;&gt;"",$C11,$B11)))&lt;IF($E11&lt;&gt;"",IF($D11&lt;&gt;"",$D11,IF($C11&lt;&gt;"",$C11,$B11)),IF($D11&lt;&gt;"",IF($C11&lt;&gt;"",$C11,$B11),IF($C11&lt;&gt;"",$B11,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="n"/>
-      <c r="B12" s="21" t="n"/>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="17">
-        <f>IF(COUNT(B12:E12)&gt;0,AVERAGE(B12:E12),"")</f>
-        <v/>
-      </c>
-      <c r="G12" s="11">
-        <f>IF(AND(E12&lt;&gt;"",D12&lt;&gt;""),IF(E12&gt;D12,"↑ Mejora",IF(E12&lt;D12,"↓ Baja","→ Estable")),"")</f>
+      <c r="A12" s="30" t="n"/>
+      <c r="B12" s="57" t="n"/>
+      <c r="C12" s="57" t="n"/>
+      <c r="D12" s="57" t="n"/>
+      <c r="E12" s="57" t="n"/>
+      <c r="F12" s="58">
+        <f>IF(COUNT($B12:$E12)=0,"",ROUND(AVERAGE($B12:$E12),2))</f>
+        <v/>
+      </c>
+      <c r="G12" s="34">
+        <f>IF(COUNT($B12:$E12)&lt;2,"",IF(IF($E12&lt;&gt;"",$E12,IF($D12&lt;&gt;"",$D12,IF($C12&lt;&gt;"",$C12,$B12)))&gt;IF($E12&lt;&gt;"",IF($D12&lt;&gt;"",$D12,IF($C12&lt;&gt;"",$C12,$B12)),IF($D12&lt;&gt;"",IF($C12&lt;&gt;"",$C12,$B12),IF($C12&lt;&gt;"",$B12,""))),"↑ Mejora",IF(IF($E12&lt;&gt;"",$E12,IF($D12&lt;&gt;"",$D12,IF($C12&lt;&gt;"",$C12,$B12)))&lt;IF($E12&lt;&gt;"",IF($D12&lt;&gt;"",$D12,IF($C12&lt;&gt;"",$C12,$B12)),IF($D12&lt;&gt;"",IF($C12&lt;&gt;"",$C12,$B12),IF($C12&lt;&gt;"",$B12,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="n"/>
-      <c r="B13" s="21" t="n"/>
-      <c r="C13" s="21" t="n"/>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="21" t="n"/>
-      <c r="F13" s="17">
-        <f>IF(COUNT(B13:E13)&gt;0,AVERAGE(B13:E13),"")</f>
-        <v/>
-      </c>
-      <c r="G13" s="11">
-        <f>IF(AND(E13&lt;&gt;"",D13&lt;&gt;""),IF(E13&gt;D13,"↑ Mejora",IF(E13&lt;D13,"↓ Baja","→ Estable")),"")</f>
+      <c r="A13" s="30" t="n"/>
+      <c r="B13" s="57" t="n"/>
+      <c r="C13" s="57" t="n"/>
+      <c r="D13" s="57" t="n"/>
+      <c r="E13" s="57" t="n"/>
+      <c r="F13" s="58">
+        <f>IF(COUNT($B13:$E13)=0,"",ROUND(AVERAGE($B13:$E13),2))</f>
+        <v/>
+      </c>
+      <c r="G13" s="34">
+        <f>IF(COUNT($B13:$E13)&lt;2,"",IF(IF($E13&lt;&gt;"",$E13,IF($D13&lt;&gt;"",$D13,IF($C13&lt;&gt;"",$C13,$B13)))&gt;IF($E13&lt;&gt;"",IF($D13&lt;&gt;"",$D13,IF($C13&lt;&gt;"",$C13,$B13)),IF($D13&lt;&gt;"",IF($C13&lt;&gt;"",$C13,$B13),IF($C13&lt;&gt;"",$B13,""))),"↑ Mejora",IF(IF($E13&lt;&gt;"",$E13,IF($D13&lt;&gt;"",$D13,IF($C13&lt;&gt;"",$C13,$B13)))&lt;IF($E13&lt;&gt;"",IF($D13&lt;&gt;"",$D13,IF($C13&lt;&gt;"",$C13,$B13)),IF($D13&lt;&gt;"",IF($C13&lt;&gt;"",$C13,$B13),IF($C13&lt;&gt;"",$B13,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="n"/>
-      <c r="B14" s="21" t="n"/>
-      <c r="C14" s="21" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="21" t="n"/>
-      <c r="F14" s="17">
-        <f>IF(COUNT(B14:E14)&gt;0,AVERAGE(B14:E14),"")</f>
-        <v/>
-      </c>
-      <c r="G14" s="11">
-        <f>IF(AND(E14&lt;&gt;"",D14&lt;&gt;""),IF(E14&gt;D14,"↑ Mejora",IF(E14&lt;D14,"↓ Baja","→ Estable")),"")</f>
+      <c r="A14" s="30" t="n"/>
+      <c r="B14" s="57" t="n"/>
+      <c r="C14" s="57" t="n"/>
+      <c r="D14" s="57" t="n"/>
+      <c r="E14" s="57" t="n"/>
+      <c r="F14" s="58">
+        <f>IF(COUNT($B14:$E14)=0,"",ROUND(AVERAGE($B14:$E14),2))</f>
+        <v/>
+      </c>
+      <c r="G14" s="34">
+        <f>IF(COUNT($B14:$E14)&lt;2,"",IF(IF($E14&lt;&gt;"",$E14,IF($D14&lt;&gt;"",$D14,IF($C14&lt;&gt;"",$C14,$B14)))&gt;IF($E14&lt;&gt;"",IF($D14&lt;&gt;"",$D14,IF($C14&lt;&gt;"",$C14,$B14)),IF($D14&lt;&gt;"",IF($C14&lt;&gt;"",$C14,$B14),IF($C14&lt;&gt;"",$B14,""))),"↑ Mejora",IF(IF($E14&lt;&gt;"",$E14,IF($D14&lt;&gt;"",$D14,IF($C14&lt;&gt;"",$C14,$B14)))&lt;IF($E14&lt;&gt;"",IF($D14&lt;&gt;"",$D14,IF($C14&lt;&gt;"",$C14,$B14)),IF($D14&lt;&gt;"",IF($C14&lt;&gt;"",$C14,$B14),IF($C14&lt;&gt;"",$B14,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="n"/>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="21" t="n"/>
-      <c r="D15" s="21" t="n"/>
-      <c r="E15" s="21" t="n"/>
-      <c r="F15" s="17">
-        <f>IF(COUNT(B15:E15)&gt;0,AVERAGE(B15:E15),"")</f>
-        <v/>
-      </c>
-      <c r="G15" s="11">
-        <f>IF(AND(E15&lt;&gt;"",D15&lt;&gt;""),IF(E15&gt;D15,"↑ Mejora",IF(E15&lt;D15,"↓ Baja","→ Estable")),"")</f>
+      <c r="A15" s="30" t="n"/>
+      <c r="B15" s="57" t="n"/>
+      <c r="C15" s="57" t="n"/>
+      <c r="D15" s="57" t="n"/>
+      <c r="E15" s="57" t="n"/>
+      <c r="F15" s="58">
+        <f>IF(COUNT($B15:$E15)=0,"",ROUND(AVERAGE($B15:$E15),2))</f>
+        <v/>
+      </c>
+      <c r="G15" s="34">
+        <f>IF(COUNT($B15:$E15)&lt;2,"",IF(IF($E15&lt;&gt;"",$E15,IF($D15&lt;&gt;"",$D15,IF($C15&lt;&gt;"",$C15,$B15)))&gt;IF($E15&lt;&gt;"",IF($D15&lt;&gt;"",$D15,IF($C15&lt;&gt;"",$C15,$B15)),IF($D15&lt;&gt;"",IF($C15&lt;&gt;"",$C15,$B15),IF($C15&lt;&gt;"",$B15,""))),"↑ Mejora",IF(IF($E15&lt;&gt;"",$E15,IF($D15&lt;&gt;"",$D15,IF($C15&lt;&gt;"",$C15,$B15)))&lt;IF($E15&lt;&gt;"",IF($D15&lt;&gt;"",$D15,IF($C15&lt;&gt;"",$C15,$B15)),IF($D15&lt;&gt;"",IF($C15&lt;&gt;"",$C15,$B15),IF($C15&lt;&gt;"",$B15,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="n"/>
-      <c r="B16" s="21" t="n"/>
-      <c r="C16" s="21" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="E16" s="21" t="n"/>
-      <c r="F16" s="17">
-        <f>IF(COUNT(B16:E16)&gt;0,AVERAGE(B16:E16),"")</f>
-        <v/>
-      </c>
-      <c r="G16" s="11">
-        <f>IF(AND(E16&lt;&gt;"",D16&lt;&gt;""),IF(E16&gt;D16,"↑ Mejora",IF(E16&lt;D16,"↓ Baja","→ Estable")),"")</f>
+      <c r="A16" s="30" t="n"/>
+      <c r="B16" s="57" t="n"/>
+      <c r="C16" s="57" t="n"/>
+      <c r="D16" s="57" t="n"/>
+      <c r="E16" s="57" t="n"/>
+      <c r="F16" s="58">
+        <f>IF(COUNT($B16:$E16)=0,"",ROUND(AVERAGE($B16:$E16),2))</f>
+        <v/>
+      </c>
+      <c r="G16" s="34">
+        <f>IF(COUNT($B16:$E16)&lt;2,"",IF(IF($E16&lt;&gt;"",$E16,IF($D16&lt;&gt;"",$D16,IF($C16&lt;&gt;"",$C16,$B16)))&gt;IF($E16&lt;&gt;"",IF($D16&lt;&gt;"",$D16,IF($C16&lt;&gt;"",$C16,$B16)),IF($D16&lt;&gt;"",IF($C16&lt;&gt;"",$C16,$B16),IF($C16&lt;&gt;"",$B16,""))),"↑ Mejora",IF(IF($E16&lt;&gt;"",$E16,IF($D16&lt;&gt;"",$D16,IF($C16&lt;&gt;"",$C16,$B16)))&lt;IF($E16&lt;&gt;"",IF($D16&lt;&gt;"",$D16,IF($C16&lt;&gt;"",$C16,$B16)),IF($D16&lt;&gt;"",IF($C16&lt;&gt;"",$C16,$B16),IF($C16&lt;&gt;"",$B16,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="n"/>
-      <c r="B17" s="21" t="n"/>
-      <c r="C17" s="21" t="n"/>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="21" t="n"/>
-      <c r="F17" s="17">
-        <f>IF(COUNT(B17:E17)&gt;0,AVERAGE(B17:E17),"")</f>
-        <v/>
-      </c>
-      <c r="G17" s="11">
-        <f>IF(AND(E17&lt;&gt;"",D17&lt;&gt;""),IF(E17&gt;D17,"↑ Mejora",IF(E17&lt;D17,"↓ Baja","→ Estable")),"")</f>
+      <c r="A17" s="30" t="n"/>
+      <c r="B17" s="57" t="n"/>
+      <c r="C17" s="57" t="n"/>
+      <c r="D17" s="57" t="n"/>
+      <c r="E17" s="57" t="n"/>
+      <c r="F17" s="58">
+        <f>IF(COUNT($B17:$E17)=0,"",ROUND(AVERAGE($B17:$E17),2))</f>
+        <v/>
+      </c>
+      <c r="G17" s="34">
+        <f>IF(COUNT($B17:$E17)&lt;2,"",IF(IF($E17&lt;&gt;"",$E17,IF($D17&lt;&gt;"",$D17,IF($C17&lt;&gt;"",$C17,$B17)))&gt;IF($E17&lt;&gt;"",IF($D17&lt;&gt;"",$D17,IF($C17&lt;&gt;"",$C17,$B17)),IF($D17&lt;&gt;"",IF($C17&lt;&gt;"",$C17,$B17),IF($C17&lt;&gt;"",$B17,""))),"↑ Mejora",IF(IF($E17&lt;&gt;"",$E17,IF($D17&lt;&gt;"",$D17,IF($C17&lt;&gt;"",$C17,$B17)))&lt;IF($E17&lt;&gt;"",IF($D17&lt;&gt;"",$D17,IF($C17&lt;&gt;"",$C17,$B17)),IF($D17&lt;&gt;"",IF($C17&lt;&gt;"",$C17,$B17),IF($C17&lt;&gt;"",$B17,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="n"/>
-      <c r="B18" s="21" t="n"/>
-      <c r="C18" s="21" t="n"/>
-      <c r="D18" s="21" t="n"/>
-      <c r="E18" s="21" t="n"/>
-      <c r="F18" s="17">
-        <f>IF(COUNT(B18:E18)&gt;0,AVERAGE(B18:E18),"")</f>
-        <v/>
-      </c>
-      <c r="G18" s="11">
-        <f>IF(AND(E18&lt;&gt;"",D18&lt;&gt;""),IF(E18&gt;D18,"↑ Mejora",IF(E18&lt;D18,"↓ Baja","→ Estable")),"")</f>
+      <c r="A18" s="30" t="n"/>
+      <c r="B18" s="57" t="n"/>
+      <c r="C18" s="57" t="n"/>
+      <c r="D18" s="57" t="n"/>
+      <c r="E18" s="57" t="n"/>
+      <c r="F18" s="58">
+        <f>IF(COUNT($B18:$E18)=0,"",ROUND(AVERAGE($B18:$E18),2))</f>
+        <v/>
+      </c>
+      <c r="G18" s="34">
+        <f>IF(COUNT($B18:$E18)&lt;2,"",IF(IF($E18&lt;&gt;"",$E18,IF($D18&lt;&gt;"",$D18,IF($C18&lt;&gt;"",$C18,$B18)))&gt;IF($E18&lt;&gt;"",IF($D18&lt;&gt;"",$D18,IF($C18&lt;&gt;"",$C18,$B18)),IF($D18&lt;&gt;"",IF($C18&lt;&gt;"",$C18,$B18),IF($C18&lt;&gt;"",$B18,""))),"↑ Mejora",IF(IF($E18&lt;&gt;"",$E18,IF($D18&lt;&gt;"",$D18,IF($C18&lt;&gt;"",$C18,$B18)))&lt;IF($E18&lt;&gt;"",IF($D18&lt;&gt;"",$D18,IF($C18&lt;&gt;"",$C18,$B18)),IF($D18&lt;&gt;"",IF($C18&lt;&gt;"",$C18,$B18),IF($C18&lt;&gt;"",$B18,""))),"↓ Baja","→ Estable")))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="n"/>
-      <c r="B19" s="21" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="21" t="n"/>
-      <c r="E19" s="21" t="n"/>
-      <c r="F19" s="17">
-        <f>IF(COUNT(B19:E19)&gt;0,AVERAGE(B19:E19),"")</f>
-        <v/>
-      </c>
-      <c r="G19" s="11">
-        <f>IF(AND(E19&lt;&gt;"",D19&lt;&gt;""),IF(E19&gt;D19,"↑ Mejora",IF(E19&lt;D19,"↓ Baja","→ Estable")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21"/>
+      <c r="A19" s="30" t="n"/>
+      <c r="B19" s="57" t="n"/>
+      <c r="C19" s="57" t="n"/>
+      <c r="D19" s="57" t="n"/>
+      <c r="E19" s="57" t="n"/>
+      <c r="F19" s="58">
+        <f>IF(COUNT($B19:$E19)=0,"",ROUND(AVERAGE($B19:$E19),2))</f>
+        <v/>
+      </c>
+      <c r="G19" s="34">
+        <f>IF(COUNT($B19:$E19)&lt;2,"",IF(IF($E19&lt;&gt;"",$E19,IF($D19&lt;&gt;"",$D19,IF($C19&lt;&gt;"",$C19,$B19)))&gt;IF($E19&lt;&gt;"",IF($D19&lt;&gt;"",$D19,IF($C19&lt;&gt;"",$C19,$B19)),IF($D19&lt;&gt;"",IF($C19&lt;&gt;"",$C19,$B19),IF($C19&lt;&gt;"",$B19,""))),"↑ Mejora",IF(IF($E19&lt;&gt;"",$E19,IF($D19&lt;&gt;"",$D19,IF($C19&lt;&gt;"",$C19,$B19)))&lt;IF($E19&lt;&gt;"",IF($D19&lt;&gt;"",$D19,IF($C19&lt;&gt;"",$C19,$B19)),IF($D19&lt;&gt;"",IF($C19&lt;&gt;"",$C19,$B19),IF($C19&lt;&gt;"",$B19,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="59" t="n"/>
+      <c r="B20" s="60" t="n"/>
+      <c r="C20" s="60" t="n"/>
+      <c r="D20" s="60" t="n"/>
+      <c r="E20" s="60" t="n"/>
+      <c r="F20" s="61">
+        <f>IF(COUNT($B20:$E20)=0,"",ROUND(AVERAGE($B20:$E20),2))</f>
+        <v/>
+      </c>
+      <c r="G20" s="43">
+        <f>IF(COUNT($B20:$E20)&lt;2,"",IF(IF($E20&lt;&gt;"",$E20,IF($D20&lt;&gt;"",$D20,IF($C20&lt;&gt;"",$C20,$B20)))&gt;IF($E20&lt;&gt;"",IF($D20&lt;&gt;"",$D20,IF($C20&lt;&gt;"",$C20,$B20)),IF($D20&lt;&gt;"",IF($C20&lt;&gt;"",$C20,$B20),IF($C20&lt;&gt;"",$B20,""))),"↑ Mejora",IF(IF($E20&lt;&gt;"",$E20,IF($D20&lt;&gt;"",$D20,IF($C20&lt;&gt;"",$C20,$B20)))&lt;IF($E20&lt;&gt;"",IF($D20&lt;&gt;"",$D20,IF($C20&lt;&gt;"",$C20,$B20)),IF($D20&lt;&gt;"",IF($C20&lt;&gt;"",$C20,$B20),IF($C20&lt;&gt;"",$B20,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="59" t="n"/>
+      <c r="B21" s="60" t="n"/>
+      <c r="C21" s="60" t="n"/>
+      <c r="D21" s="60" t="n"/>
+      <c r="E21" s="60" t="n"/>
+      <c r="F21" s="61">
+        <f>IF(COUNT($B21:$E21)=0,"",ROUND(AVERAGE($B21:$E21),2))</f>
+        <v/>
+      </c>
+      <c r="G21" s="43">
+        <f>IF(COUNT($B21:$E21)&lt;2,"",IF(IF($E21&lt;&gt;"",$E21,IF($D21&lt;&gt;"",$D21,IF($C21&lt;&gt;"",$C21,$B21)))&gt;IF($E21&lt;&gt;"",IF($D21&lt;&gt;"",$D21,IF($C21&lt;&gt;"",$C21,$B21)),IF($D21&lt;&gt;"",IF($C21&lt;&gt;"",$C21,$B21),IF($C21&lt;&gt;"",$B21,""))),"↑ Mejora",IF(IF($E21&lt;&gt;"",$E21,IF($D21&lt;&gt;"",$D21,IF($C21&lt;&gt;"",$C21,$B21)))&lt;IF($E21&lt;&gt;"",IF($D21&lt;&gt;"",$D21,IF($C21&lt;&gt;"",$C21,$B21)),IF($D21&lt;&gt;"",IF($C21&lt;&gt;"",$C21,$B21),IF($C21&lt;&gt;"",$B21,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="59" t="n"/>
+      <c r="B22" s="60" t="n"/>
+      <c r="C22" s="60" t="n"/>
+      <c r="D22" s="60" t="n"/>
+      <c r="E22" s="60" t="n"/>
+      <c r="F22" s="61">
+        <f>IF(COUNT($B22:$E22)=0,"",ROUND(AVERAGE($B22:$E22),2))</f>
+        <v/>
+      </c>
+      <c r="G22" s="43">
+        <f>IF(COUNT($B22:$E22)&lt;2,"",IF(IF($E22&lt;&gt;"",$E22,IF($D22&lt;&gt;"",$D22,IF($C22&lt;&gt;"",$C22,$B22)))&gt;IF($E22&lt;&gt;"",IF($D22&lt;&gt;"",$D22,IF($C22&lt;&gt;"",$C22,$B22)),IF($D22&lt;&gt;"",IF($C22&lt;&gt;"",$C22,$B22),IF($C22&lt;&gt;"",$B22,""))),"↑ Mejora",IF(IF($E22&lt;&gt;"",$E22,IF($D22&lt;&gt;"",$D22,IF($C22&lt;&gt;"",$C22,$B22)))&lt;IF($E22&lt;&gt;"",IF($D22&lt;&gt;"",$D22,IF($C22&lt;&gt;"",$C22,$B22)),IF($D22&lt;&gt;"",IF($C22&lt;&gt;"",$C22,$B22),IF($C22&lt;&gt;"",$B22,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="52" t="n"/>
+      <c r="B23" s="62" t="n"/>
+      <c r="C23" s="62" t="n"/>
+      <c r="D23" s="62" t="n"/>
+      <c r="E23" s="62" t="n"/>
+      <c r="F23" s="63">
+        <f>IF(COUNT($B23:$E23)=0,"",ROUND(AVERAGE($B23:$E23),2))</f>
+        <v/>
+      </c>
+      <c r="G23" s="48">
+        <f>IF(COUNT($B23:$E23)&lt;2,"",IF(IF($E23&lt;&gt;"",$E23,IF($D23&lt;&gt;"",$D23,IF($C23&lt;&gt;"",$C23,$B23)))&gt;IF($E23&lt;&gt;"",IF($D23&lt;&gt;"",$D23,IF($C23&lt;&gt;"",$C23,$B23)),IF($D23&lt;&gt;"",IF($C23&lt;&gt;"",$C23,$B23),IF($C23&lt;&gt;"",$B23,""))),"↑ Mejora",IF(IF($E23&lt;&gt;"",$E23,IF($D23&lt;&gt;"",$D23,IF($C23&lt;&gt;"",$C23,$B23)))&lt;IF($E23&lt;&gt;"",IF($D23&lt;&gt;"",$D23,IF($C23&lt;&gt;"",$C23,$B23)),IF($D23&lt;&gt;"",IF($C23&lt;&gt;"",$C23,$B23),IF($C23&lt;&gt;"",$B23,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="52" t="n"/>
+      <c r="B24" s="62" t="n"/>
+      <c r="C24" s="62" t="n"/>
+      <c r="D24" s="62" t="n"/>
+      <c r="E24" s="62" t="n"/>
+      <c r="F24" s="63">
+        <f>IF(COUNT($B24:$E24)=0,"",ROUND(AVERAGE($B24:$E24),2))</f>
+        <v/>
+      </c>
+      <c r="G24" s="48">
+        <f>IF(COUNT($B24:$E24)&lt;2,"",IF(IF($E24&lt;&gt;"",$E24,IF($D24&lt;&gt;"",$D24,IF($C24&lt;&gt;"",$C24,$B24)))&gt;IF($E24&lt;&gt;"",IF($D24&lt;&gt;"",$D24,IF($C24&lt;&gt;"",$C24,$B24)),IF($D24&lt;&gt;"",IF($C24&lt;&gt;"",$C24,$B24),IF($C24&lt;&gt;"",$B24,""))),"↑ Mejora",IF(IF($E24&lt;&gt;"",$E24,IF($D24&lt;&gt;"",$D24,IF($C24&lt;&gt;"",$C24,$B24)))&lt;IF($E24&lt;&gt;"",IF($D24&lt;&gt;"",$D24,IF($C24&lt;&gt;"",$C24,$B24)),IF($D24&lt;&gt;"",IF($C24&lt;&gt;"",$C24,$B24),IF($C24&lt;&gt;"",$B24,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="52" t="n"/>
+      <c r="B25" s="62" t="n"/>
+      <c r="C25" s="62" t="n"/>
+      <c r="D25" s="62" t="n"/>
+      <c r="E25" s="62" t="n"/>
+      <c r="F25" s="63">
+        <f>IF(COUNT($B25:$E25)=0,"",ROUND(AVERAGE($B25:$E25),2))</f>
+        <v/>
+      </c>
+      <c r="G25" s="48">
+        <f>IF(COUNT($B25:$E25)&lt;2,"",IF(IF($E25&lt;&gt;"",$E25,IF($D25&lt;&gt;"",$D25,IF($C25&lt;&gt;"",$C25,$B25)))&gt;IF($E25&lt;&gt;"",IF($D25&lt;&gt;"",$D25,IF($C25&lt;&gt;"",$C25,$B25)),IF($D25&lt;&gt;"",IF($C25&lt;&gt;"",$C25,$B25),IF($C25&lt;&gt;"",$B25,""))),"↑ Mejora",IF(IF($E25&lt;&gt;"",$E25,IF($D25&lt;&gt;"",$D25,IF($C25&lt;&gt;"",$C25,$B25)))&lt;IF($E25&lt;&gt;"",IF($D25&lt;&gt;"",$D25,IF($C25&lt;&gt;"",$C25,$B25)),IF($D25&lt;&gt;"",IF($C25&lt;&gt;"",$C25,$B25),IF($C25&lt;&gt;"",$B25,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="52" t="n"/>
+      <c r="B26" s="62" t="n"/>
+      <c r="C26" s="62" t="n"/>
+      <c r="D26" s="62" t="n"/>
+      <c r="E26" s="62" t="n"/>
+      <c r="F26" s="63">
+        <f>IF(COUNT($B26:$E26)=0,"",ROUND(AVERAGE($B26:$E26),2))</f>
+        <v/>
+      </c>
+      <c r="G26" s="48">
+        <f>IF(COUNT($B26:$E26)&lt;2,"",IF(IF($E26&lt;&gt;"",$E26,IF($D26&lt;&gt;"",$D26,IF($C26&lt;&gt;"",$C26,$B26)))&gt;IF($E26&lt;&gt;"",IF($D26&lt;&gt;"",$D26,IF($C26&lt;&gt;"",$C26,$B26)),IF($D26&lt;&gt;"",IF($C26&lt;&gt;"",$C26,$B26),IF($C26&lt;&gt;"",$B26,""))),"↑ Mejora",IF(IF($E26&lt;&gt;"",$E26,IF($D26&lt;&gt;"",$D26,IF($C26&lt;&gt;"",$C26,$B26)))&lt;IF($E26&lt;&gt;"",IF($D26&lt;&gt;"",$D26,IF($C26&lt;&gt;"",$C26,$B26)),IF($D26&lt;&gt;"",IF($C26&lt;&gt;"",$C26,$B26),IF($C26&lt;&gt;"",$B26,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="52" t="n"/>
+      <c r="B27" s="62" t="n"/>
+      <c r="C27" s="62" t="n"/>
+      <c r="D27" s="62" t="n"/>
+      <c r="E27" s="62" t="n"/>
+      <c r="F27" s="63">
+        <f>IF(COUNT($B27:$E27)=0,"",ROUND(AVERAGE($B27:$E27),2))</f>
+        <v/>
+      </c>
+      <c r="G27" s="48">
+        <f>IF(COUNT($B27:$E27)&lt;2,"",IF(IF($E27&lt;&gt;"",$E27,IF($D27&lt;&gt;"",$D27,IF($C27&lt;&gt;"",$C27,$B27)))&gt;IF($E27&lt;&gt;"",IF($D27&lt;&gt;"",$D27,IF($C27&lt;&gt;"",$C27,$B27)),IF($D27&lt;&gt;"",IF($C27&lt;&gt;"",$C27,$B27),IF($C27&lt;&gt;"",$B27,""))),"↑ Mejora",IF(IF($E27&lt;&gt;"",$E27,IF($D27&lt;&gt;"",$D27,IF($C27&lt;&gt;"",$C27,$B27)))&lt;IF($E27&lt;&gt;"",IF($D27&lt;&gt;"",$D27,IF($C27&lt;&gt;"",$C27,$B27)),IF($D27&lt;&gt;"",IF($C27&lt;&gt;"",$C27,$B27),IF($C27&lt;&gt;"",$B27,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="52" t="n"/>
+      <c r="B28" s="62" t="n"/>
+      <c r="C28" s="62" t="n"/>
+      <c r="D28" s="62" t="n"/>
+      <c r="E28" s="62" t="n"/>
+      <c r="F28" s="63">
+        <f>IF(COUNT($B28:$E28)=0,"",ROUND(AVERAGE($B28:$E28),2))</f>
+        <v/>
+      </c>
+      <c r="G28" s="48">
+        <f>IF(COUNT($B28:$E28)&lt;2,"",IF(IF($E28&lt;&gt;"",$E28,IF($D28&lt;&gt;"",$D28,IF($C28&lt;&gt;"",$C28,$B28)))&gt;IF($E28&lt;&gt;"",IF($D28&lt;&gt;"",$D28,IF($C28&lt;&gt;"",$C28,$B28)),IF($D28&lt;&gt;"",IF($C28&lt;&gt;"",$C28,$B28),IF($C28&lt;&gt;"",$B28,""))),"↑ Mejora",IF(IF($E28&lt;&gt;"",$E28,IF($D28&lt;&gt;"",$D28,IF($C28&lt;&gt;"",$C28,$B28)))&lt;IF($E28&lt;&gt;"",IF($D28&lt;&gt;"",$D28,IF($C28&lt;&gt;"",$C28,$B28)),IF($D28&lt;&gt;"",IF($C28&lt;&gt;"",$C28,$B28),IF($C28&lt;&gt;"",$B28,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="52" t="n"/>
+      <c r="B29" s="62" t="n"/>
+      <c r="C29" s="62" t="n"/>
+      <c r="D29" s="62" t="n"/>
+      <c r="E29" s="62" t="n"/>
+      <c r="F29" s="63">
+        <f>IF(COUNT($B29:$E29)=0,"",ROUND(AVERAGE($B29:$E29),2))</f>
+        <v/>
+      </c>
+      <c r="G29" s="48">
+        <f>IF(COUNT($B29:$E29)&lt;2,"",IF(IF($E29&lt;&gt;"",$E29,IF($D29&lt;&gt;"",$D29,IF($C29&lt;&gt;"",$C29,$B29)))&gt;IF($E29&lt;&gt;"",IF($D29&lt;&gt;"",$D29,IF($C29&lt;&gt;"",$C29,$B29)),IF($D29&lt;&gt;"",IF($C29&lt;&gt;"",$C29,$B29),IF($C29&lt;&gt;"",$B29,""))),"↑ Mejora",IF(IF($E29&lt;&gt;"",$E29,IF($D29&lt;&gt;"",$D29,IF($C29&lt;&gt;"",$C29,$B29)))&lt;IF($E29&lt;&gt;"",IF($D29&lt;&gt;"",$D29,IF($C29&lt;&gt;"",$C29,$B29)),IF($D29&lt;&gt;"",IF($C29&lt;&gt;"",$C29,$B29),IF($C29&lt;&gt;"",$B29,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="52" t="n"/>
+      <c r="B30" s="62" t="n"/>
+      <c r="C30" s="62" t="n"/>
+      <c r="D30" s="62" t="n"/>
+      <c r="E30" s="62" t="n"/>
+      <c r="F30" s="63">
+        <f>IF(COUNT($B30:$E30)=0,"",ROUND(AVERAGE($B30:$E30),2))</f>
+        <v/>
+      </c>
+      <c r="G30" s="48">
+        <f>IF(COUNT($B30:$E30)&lt;2,"",IF(IF($E30&lt;&gt;"",$E30,IF($D30&lt;&gt;"",$D30,IF($C30&lt;&gt;"",$C30,$B30)))&gt;IF($E30&lt;&gt;"",IF($D30&lt;&gt;"",$D30,IF($C30&lt;&gt;"",$C30,$B30)),IF($D30&lt;&gt;"",IF($C30&lt;&gt;"",$C30,$B30),IF($C30&lt;&gt;"",$B30,""))),"↑ Mejora",IF(IF($E30&lt;&gt;"",$E30,IF($D30&lt;&gt;"",$D30,IF($C30&lt;&gt;"",$C30,$B30)))&lt;IF($E30&lt;&gt;"",IF($D30&lt;&gt;"",$D30,IF($C30&lt;&gt;"",$C30,$B30)),IF($D30&lt;&gt;"",IF($C30&lt;&gt;"",$C30,$B30),IF($C30&lt;&gt;"",$B30,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="52" t="n"/>
+      <c r="B31" s="62" t="n"/>
+      <c r="C31" s="62" t="n"/>
+      <c r="D31" s="62" t="n"/>
+      <c r="E31" s="62" t="n"/>
+      <c r="F31" s="63">
+        <f>IF(COUNT($B31:$E31)=0,"",ROUND(AVERAGE($B31:$E31),2))</f>
+        <v/>
+      </c>
+      <c r="G31" s="48">
+        <f>IF(COUNT($B31:$E31)&lt;2,"",IF(IF($E31&lt;&gt;"",$E31,IF($D31&lt;&gt;"",$D31,IF($C31&lt;&gt;"",$C31,$B31)))&gt;IF($E31&lt;&gt;"",IF($D31&lt;&gt;"",$D31,IF($C31&lt;&gt;"",$C31,$B31)),IF($D31&lt;&gt;"",IF($C31&lt;&gt;"",$C31,$B31),IF($C31&lt;&gt;"",$B31,""))),"↑ Mejora",IF(IF($E31&lt;&gt;"",$E31,IF($D31&lt;&gt;"",$D31,IF($C31&lt;&gt;"",$C31,$B31)))&lt;IF($E31&lt;&gt;"",IF($D31&lt;&gt;"",$D31,IF($C31&lt;&gt;"",$C31,$B31)),IF($D31&lt;&gt;"",IF($C31&lt;&gt;"",$C31,$B31),IF($C31&lt;&gt;"",$B31,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="52" t="n"/>
+      <c r="B32" s="62" t="n"/>
+      <c r="C32" s="62" t="n"/>
+      <c r="D32" s="62" t="n"/>
+      <c r="E32" s="62" t="n"/>
+      <c r="F32" s="63">
+        <f>IF(COUNT($B32:$E32)=0,"",ROUND(AVERAGE($B32:$E32),2))</f>
+        <v/>
+      </c>
+      <c r="G32" s="48">
+        <f>IF(COUNT($B32:$E32)&lt;2,"",IF(IF($E32&lt;&gt;"",$E32,IF($D32&lt;&gt;"",$D32,IF($C32&lt;&gt;"",$C32,$B32)))&gt;IF($E32&lt;&gt;"",IF($D32&lt;&gt;"",$D32,IF($C32&lt;&gt;"",$C32,$B32)),IF($D32&lt;&gt;"",IF($C32&lt;&gt;"",$C32,$B32),IF($C32&lt;&gt;"",$B32,""))),"↑ Mejora",IF(IF($E32&lt;&gt;"",$E32,IF($D32&lt;&gt;"",$D32,IF($C32&lt;&gt;"",$C32,$B32)))&lt;IF($E32&lt;&gt;"",IF($D32&lt;&gt;"",$D32,IF($C32&lt;&gt;"",$C32,$B32)),IF($D32&lt;&gt;"",IF($C32&lt;&gt;"",$C32,$B32),IF($C32&lt;&gt;"",$B32,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="52" t="n"/>
+      <c r="B33" s="62" t="n"/>
+      <c r="C33" s="62" t="n"/>
+      <c r="D33" s="62" t="n"/>
+      <c r="E33" s="62" t="n"/>
+      <c r="F33" s="63">
+        <f>IF(COUNT($B33:$E33)=0,"",ROUND(AVERAGE($B33:$E33),2))</f>
+        <v/>
+      </c>
+      <c r="G33" s="48">
+        <f>IF(COUNT($B33:$E33)&lt;2,"",IF(IF($E33&lt;&gt;"",$E33,IF($D33&lt;&gt;"",$D33,IF($C33&lt;&gt;"",$C33,$B33)))&gt;IF($E33&lt;&gt;"",IF($D33&lt;&gt;"",$D33,IF($C33&lt;&gt;"",$C33,$B33)),IF($D33&lt;&gt;"",IF($C33&lt;&gt;"",$C33,$B33),IF($C33&lt;&gt;"",$B33,""))),"↑ Mejora",IF(IF($E33&lt;&gt;"",$E33,IF($D33&lt;&gt;"",$D33,IF($C33&lt;&gt;"",$C33,$B33)))&lt;IF($E33&lt;&gt;"",IF($D33&lt;&gt;"",$D33,IF($C33&lt;&gt;"",$C33,$B33)),IF($D33&lt;&gt;"",IF($C33&lt;&gt;"",$C33,$B33),IF($C33&lt;&gt;"",$B33,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="52" t="n"/>
+      <c r="B34" s="62" t="n"/>
+      <c r="C34" s="62" t="n"/>
+      <c r="D34" s="62" t="n"/>
+      <c r="E34" s="62" t="n"/>
+      <c r="F34" s="63">
+        <f>IF(COUNT($B34:$E34)=0,"",ROUND(AVERAGE($B34:$E34),2))</f>
+        <v/>
+      </c>
+      <c r="G34" s="48">
+        <f>IF(COUNT($B34:$E34)&lt;2,"",IF(IF($E34&lt;&gt;"",$E34,IF($D34&lt;&gt;"",$D34,IF($C34&lt;&gt;"",$C34,$B34)))&gt;IF($E34&lt;&gt;"",IF($D34&lt;&gt;"",$D34,IF($C34&lt;&gt;"",$C34,$B34)),IF($D34&lt;&gt;"",IF($C34&lt;&gt;"",$C34,$B34),IF($C34&lt;&gt;"",$B34,""))),"↑ Mejora",IF(IF($E34&lt;&gt;"",$E34,IF($D34&lt;&gt;"",$D34,IF($C34&lt;&gt;"",$C34,$B34)))&lt;IF($E34&lt;&gt;"",IF($D34&lt;&gt;"",$D34,IF($C34&lt;&gt;"",$C34,$B34)),IF($D34&lt;&gt;"",IF($C34&lt;&gt;"",$C34,$B34),IF($C34&lt;&gt;"",$B34,""))),"↓ Baja","→ Estable")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="64" t="inlineStr">
+        <is>
+          <t>▸ Vuelca aquí la PUNTUACIÓN MEDIA (celda C22) de cada ficha: una columna por trimestre y una fila por empleado. La Tendencia compara los DOS ÚLTIMOS trimestres informados aunque haya huecos en medio: si evalúas dos veces al año, deja los trimestres que no toques en blanco y la comparación sigue siendo la correcta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="64" t="inlineStr">
+        <is>
+          <t>▸ «Media Anual» se queda en blanco mientras no haya ni una nota: un empleado sin evaluar no es un empleado con un cero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="64" t="inlineStr">
+        <is>
+          <t>▸ La hoja admite 30 empleados, los mismos que el directorio (07) y que el cuadrante (01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="51" t="inlineStr">
         <is>
           <t>© 2026 AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A22:G22"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="6">
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A38:G38"/>
   </mergeCells>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>